<commit_message>
updates for sentence splitting, closes #25
</commit_message>
<xml_diff>
--- a/ready-for-annotation/de/teddy-4929.xlsx
+++ b/ready-for-annotation/de/teddy-4929.xlsx
@@ -62,7 +62,7 @@
     <t>Mai 1941 sank das deutsche Schlachtschiff Bismarck in einem heftigen Feuergefecht .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s2_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s2_0</t>
   </si>
   <si>
     <t>6</t>
@@ -74,7 +74,7 @@
     <t>Nur 118 der 2.200 Besatzungsmitglieder überlebten .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s3_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s3_0</t>
   </si>
   <si>
     <t>4</t>
@@ -89,7 +89,7 @@
     <t>Aber als ein britischer Zerstörer die Gefangenen aufnahm , fand man einen unerwarteten Überlebenden : eine schwarzweiße Katze , die sich an eine Planke klammerte .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s4_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s4_0</t>
   </si>
   <si>
     <t>5</t>
@@ -101,7 +101,7 @@
     <t>In den Folgemonaten fing die Katze Ratten und hob die Moral der Briten , bis das Schiff von einem Torpedo getroffen wurde und sank .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s5_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s5_0</t>
   </si>
   <si>
     <t>bleiben</t>
@@ -110,7 +110,7 @@
     <t>Doch wie durch ein Wunder blieb die Katze am an dem Leben .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s6_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s6_0</t>
   </si>
   <si>
     <t>7</t>
@@ -122,7 +122,7 @@
     <t>Sie wurde &amp;quot; Unsinkbarer Sam &amp;quot; getauft , fuhr mit der geretteten Crew nach Gibraltar und diente auf drei anderen Schiffen , von denen ein weiteres sank , bevor sie sich im in dem Belfaster Heim für Seeleute zur zu der Ruhe setzte .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s7_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s7_0</t>
   </si>
   <si>
     <t>8</t>
@@ -134,7 +134,7 @@
     <t>Viele sehen Katzen wohl nicht als taugliche Matrosen oder kooperative Begleiter jeglicher Art .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s8_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s8_0</t>
   </si>
   <si>
     <t>9</t>
@@ -146,7 +146,7 @@
     <t>Aber Katzen arbeiten seit Jahrtausenden mit uns Menschen zusammen und helfen uns so oft wie wir ihnen .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s9_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s9_0</t>
   </si>
   <si>
     <t>werden</t>
@@ -155,7 +155,7 @@
     <t>Wie wurden diese Einzelgänger vom von dem wilden Raubtier zum zu dem Marineoffizier und Couchgenossen ?</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s10_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s10_0</t>
   </si>
   <si>
     <t>11</t>
@@ -167,7 +167,7 @@
     <t>Die Domestizierung der modernen Hauskatze lässt sich im in dem Fruchtbaren Halbmond über 10.000 Jahre bis zum zu dem Beginn der Jungsteinzeit zurückverfolgen .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s11_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s11_0</t>
   </si>
   <si>
     <t>12</t>
@@ -179,7 +179,7 @@
     <t>Die Menschen zähmten die Natur und produzierten mehr Nahrung , als sie essen konnten .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s12_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s12_0</t>
   </si>
   <si>
     <t>13</t>
@@ -191,7 +191,7 @@
     <t>Sie lagerten ihr überschüssiges Korn in großen Gruben und niedrigen Lehmsilos .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s13_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s13_0</t>
   </si>
   <si>
     <t>14</t>
@@ -203,7 +203,7 @@
     <t>Aber diese Lager zogen Scharen von Nagetieren und deren Jäger an Felis silvestris lybica , die Wildkatze , die in Nordafrika und Südwestasien heimisch war .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s14_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s14_0</t>
   </si>
   <si>
     <t>15</t>
@@ -215,7 +215,7 @@
     <t>Wildkatzen waren schnelle , gnadenlose Jäger und unserer heutigen Hauskatze in Größe und Aussehen sehr ähnlich .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s15_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s15_0</t>
   </si>
   <si>
     <t>16</t>
@@ -227,7 +227,7 @@
     <t>Doch die frühere Wildkatze hatte ein gestreiftes Fell , war muskulöser und distanzierter gegenüber anderen Katzen und Menschen .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s16_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s16_0</t>
   </si>
   <si>
     <t>17</t>
@@ -239,7 +239,7 @@
     <t>Die Beutemenge in den Kornspeichern lockte die typischen Einzelgänger an .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s17_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s17_0</t>
   </si>
   <si>
     <t>18</t>
@@ -251,7 +251,7 @@
     <t>Als sich die Wildkatzen beim bei dem Fressen an Menschen und andere Katzen gewöhnten , tolerierten wohl auch die Bauern Katzen aufgrund der kostenlosen Schädlingsbekämpfung .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s18_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s18_0</t>
   </si>
   <si>
     <t>19</t>
@@ -263,7 +263,7 @@
     <t>Diese Beziehung war so vorteilhaft , dass die Katzen mit den Steinzeitbauern von Anatolien nach Europa und in den Mittelmeerraum auswanderten .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s19_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s19_0</t>
   </si>
   <si>
     <t>20</t>
@@ -275,7 +275,7 @@
     <t>Schädlinge waren eine Plage der Seefahrt .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s20_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s20_0</t>
   </si>
   <si>
     <t>21</t>
@@ -287,7 +287,7 @@
     <t>Sie fraßen Vorräte und nagten Taue an .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s21_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s21_0</t>
   </si>
   <si>
     <t>22</t>
@@ -299,7 +299,7 @@
     <t>Deswegen waren Katzen längst unersetzliche Schiffskumpane geworden .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s22_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s22_0</t>
   </si>
   <si>
     <t>23</t>
@@ -311,7 +311,7 @@
     <t>Ungefähr zur zu der selben Zeit , als die anatolischen Katzen Segel setzten , domestizierten die Ägypter ihre eigenen heimischen Katzen .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s23_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s23_0</t>
   </si>
   <si>
     <t>24</t>
@@ -323,7 +323,7 @@
     <t>Man verehrte sie , weil sie Giftschlangen erlegten , Vögel fingen und Ratten töteten .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s24_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s24_0</t>
   </si>
   <si>
     <t>25</t>
@@ -335,7 +335,7 @@
     <t>So erlangten Katzen Bedeutung für die ägyptische Religion .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s25_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s25_0</t>
   </si>
   <si>
     <t>26</t>
@@ -347,7 +347,7 @@
     <t>Sie wurden unsterblich durch Fresken , Hieroglyphen , Statuen und sogar Gräber , wo sie mit ihren Besitzern mumifiziert wurden .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s26_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s26_0</t>
   </si>
   <si>
     <t>27</t>
@@ -359,7 +359,7 @@
     <t>Ägyptische Schiffskatzen befuhren den Nil und hielten giftige Flussschlangen fern .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s27_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s27_0</t>
   </si>
   <si>
     <t>28</t>
@@ -371,7 +371,7 @@
     <t>Später stiegen sie auf größere Schiffe um und segelten von Hafen zu Hafen .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s28_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s28_0</t>
   </si>
   <si>
     <t>30</t>
@@ -383,7 +383,7 @@
     <t>Jahrhunderte später , im in dem Mittelalter , fuhren ägyptische Katzen auf Schiffen der Wikinger bis in die Ostsee .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s30_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s30_0</t>
   </si>
   <si>
     <t>31</t>
@@ -395,7 +395,7 @@
     <t>Sowohl nahöstliche als auch nordafrikanische Wildkatzen , damals vermutlich bereits zahm , reisten weiter quer durch Europa und setzten schließlich Segel nach Australien und Amerika .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s31_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s31_0</t>
   </si>
   <si>
     <t>32</t>
@@ -407,7 +407,7 @@
     <t>Heute stammen die meisten Hauskatzen von der nahöstlichen oder ägyptischen Linie von F. s. lybica ab .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s32_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s32_0</t>
   </si>
   <si>
     <t>33</t>
@@ -419,7 +419,7 @@
     <t>Aber genaue Analysen der Genome und Fellmuster moderner Katzen verraten :</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s33_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s33_0</t>
   </si>
   <si>
     <t>35</t>
@@ -431,7 +431,7 @@
     <t>Wir haben sie zwar sozialer und fügsamer gemacht , aber ihr natürliches Verhalten hat sich kaum verändert .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s35_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s35_0</t>
   </si>
   <si>
     <t>36</t>
@@ -443,7 +443,7 @@
     <t>Anders gesagt : Katzen von heute sind in etwa , was sie immer waren : Wildtiere .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s36_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s36_0</t>
   </si>
   <si>
     <t>37</t>
@@ -458,7 +458,7 @@
     <t>Gnadenlose Jäger .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s37_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s37_0</t>
   </si>
   <si>
     <t>38</t>
@@ -470,7 +470,7 @@
     <t>Geschöpfe , die uns nicht als ihre Halter sehen .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s38_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s38_0</t>
   </si>
   <si>
     <t>39</t>
@@ -479,7 +479,7 @@
     <t>Angesichts unserer langen gemeinsamen Geschichte haben sie wohl recht .</t>
   </si>
   <si>
-    <t>file://conllu/de/4929.conllu#s39_0</t>
+    <t>file://conllu/de/teddy-4929.conllu#s39_0</t>
   </si>
   <si>
     <t>WORD</t>

</xml_diff>